<commit_message>
Add CB Replenishment module (API + service + UI + input files)
</commit_message>
<xml_diff>
--- a/data/input/China reorder.xlsx
+++ b/data/input/China reorder.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D82D4AD9-831C-488D-9238-FD3D392C7738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C28743D-B048-4CBC-90B5-C39094B03230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E6F3F26F-327D-42FE-B92F-B9D43C18F440}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
   <si>
     <t>Avg</t>
   </si>
@@ -76,6 +77,12 @@
   </si>
   <si>
     <t>Done</t>
+  </si>
+  <si>
+    <t>CB Sales</t>
+  </si>
+  <si>
+    <t>Discussion with Kanwal - CB &amp; AA (+Tonor)</t>
   </si>
 </sst>
 </file>
@@ -450,9 +457,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{958B32DC-7C95-4B7C-A72E-304EBE582642}">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="2" max="2" width="36.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="10.5546875" customWidth="1"/>
     <col min="9" max="9" width="28.77734375" bestFit="1" customWidth="1"/>
@@ -582,6 +590,14 @@
         <v>5</v>
       </c>
     </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: CB replenishment sales window (from/to week) + cover weeks param
</commit_message>
<xml_diff>
--- a/data/input/China reorder.xlsx
+++ b/data/input/China reorder.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C28743D-B048-4CBC-90B5-C39094B03230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE6B7608-FA2F-4D7A-AD3F-752B7A72561B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E6F3F26F-327D-42FE-B92F-B9D43C18F440}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -46,12 +45,6 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>Inv less than 12 weeks mark critical</t>
-  </si>
-  <si>
-    <t>Inv between 12 to 16 weeks mark moderate</t>
-  </si>
-  <si>
     <t>More than 4 does not need reorder</t>
   </si>
   <si>
@@ -83,6 +76,12 @@
   </si>
   <si>
     <t>Discussion with Kanwal - CB &amp; AA (+Tonor)</t>
+  </si>
+  <si>
+    <t>Inv less than 18 weeks mark critical</t>
+  </si>
+  <si>
+    <t>Inv between 18 to 24 weeks mark moderate</t>
   </si>
 </sst>
 </file>
@@ -469,10 +468,10 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -509,22 +508,22 @@
         <v>114.85714285714285</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="H2" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>2</v>
@@ -537,25 +536,25 @@
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -571,7 +570,7 @@
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -587,15 +586,15 @@
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>